<commit_message>
Support flexible date parsing (YYYY-MM-DD, DD.MM.YYYY, MM/DD/YYYY)
</commit_message>
<xml_diff>
--- a/sales_report.xlsx
+++ b/sales_report.xlsx
@@ -705,7 +705,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Customer Summary  •  Generated August 15, 2026</t>
+          <t>Customer Summary  •  Generated August 16, 2026</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Full Transaction Log  •  Generated August 15, 2026</t>
+          <t>Full Transaction Log  •  Generated August 16, 2026</t>
         </is>
       </c>
     </row>

</xml_diff>